<commit_message>
Update hallucination dataset and add bar chart image
Expanded test/gpt-4o_mutation_outputs_dataset20250926_hallucination.csv with new columns and updated entries, improving data structure and clarity. Added bar_chart_square.png to test/stat/. Made updates to test/stat/calculate2.py, data.xlsx, and figure.py, and modified test/llm_prompts/prompts.py and its compiled cache. Updated slides/20251113.pptx with new content.
</commit_message>
<xml_diff>
--- a/test/stat/data.xlsx
+++ b/test/stat/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\test\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BFC7664-DD1C-40FC-9385-D66830E2C3C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{575AFDC6-936B-4DFD-B5CD-38B1E35C2726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="12">
   <si>
     <t>gpt-4o</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -68,10 +68,6 @@
   </si>
   <si>
     <t>oa-mutation</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>cove-se</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -401,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -488,6 +484,21 @@
       <c r="A6" t="s">
         <v>0</v>
       </c>
+      <c r="B6">
+        <v>12.95</v>
+      </c>
+      <c r="C6">
+        <v>88.5</v>
+      </c>
+      <c r="D6">
+        <v>14.41</v>
+      </c>
+      <c r="E6">
+        <v>1569</v>
+      </c>
+      <c r="F6">
+        <v>17.093699999999998</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -571,7 +582,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
         <v>2</v>
@@ -659,38 +670,9 @@
         <v>155.00290000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>11</v>
-      </c>
-      <c r="B21" t="s">
-        <v>2</v>
-      </c>
-      <c r="C21" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" t="s">
-        <v>4</v>
-      </c>
-      <c r="E21" t="s">
-        <v>8</v>
-      </c>
-      <c r="F21" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix question count print statement in main.py
Corrects the print statement in test/chain-of-verification-main/src/main.py to display the number of remaining questions to process (df_todo) instead of the total dataset size (df).
</commit_message>
<xml_diff>
--- a/test/stat/data.xlsx
+++ b/test/stat/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\test\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1668DA9C-764E-4B69-8C67-1249F00CA867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F235C0E0-CCF4-49CE-B07D-90EB1FA84C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="13">
   <si>
     <t>gpt-4o</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -72,6 +72,10 @@
   </si>
   <si>
     <t>cot-rag</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cove-se</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -397,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -668,6 +672,51 @@
       </c>
       <c r="F19">
         <v>155.00290000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" t="s">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D21" t="s">
+        <v>4</v>
+      </c>
+      <c r="E21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22">
+        <v>27.23</v>
+      </c>
+      <c r="C22">
+        <v>70.8</v>
+      </c>
+      <c r="D22">
+        <v>25.23</v>
+      </c>
+      <c r="E22">
+        <v>2892.71</v>
+      </c>
+      <c r="F22">
+        <v>34.570399999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update test datasets and statistical analysis scripts
Modified hallucination CSV, updated statistical figures and data files, and revised Python scripts for accuracy calculations and figure generation in the test/stat directory. These changes improve data quality and update visualizations for recent analysis results.
</commit_message>
<xml_diff>
--- a/test/stat/data.xlsx
+++ b/test/stat/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\test\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F235C0E0-CCF4-49CE-B07D-90EB1FA84C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB53D1D1-9FBB-450D-84BD-EA7024D1EAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="13">
   <si>
     <t>gpt-4o</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -43,10 +43,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>unnecessary_repair_rate</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>oa</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -76,6 +72,10 @@
   </si>
   <si>
     <t>cove-se</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>overcorrection</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -401,13 +401,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>5</v>
-      </c>
       <c r="B1" t="s">
         <v>2</v>
       </c>
@@ -415,222 +412,212 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
         <v>8</v>
-      </c>
-      <c r="F1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <v>15</v>
-      </c>
-      <c r="C2">
-        <v>85.32</v>
-      </c>
-      <c r="D2">
-        <v>17.12</v>
-      </c>
-      <c r="E2">
-        <v>289.43</v>
-      </c>
-      <c r="F2">
-        <v>1.4267000000000001</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>16.96</v>
+      </c>
+      <c r="C3">
+        <v>78.760000000000005</v>
+      </c>
+      <c r="D3">
+        <v>12.61</v>
+      </c>
+      <c r="E3">
+        <v>97.97</v>
+      </c>
+      <c r="F3">
+        <v>1.5811999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
-        <v>9.82</v>
-      </c>
-      <c r="C3">
-        <v>90.18</v>
-      </c>
-      <c r="D3">
-        <v>9.82</v>
-      </c>
-      <c r="E3">
-        <v>305.13</v>
-      </c>
-      <c r="F3">
-        <v>27.958100000000002</v>
+      <c r="B4">
+        <v>13.39</v>
+      </c>
+      <c r="C4">
+        <v>87.5</v>
+      </c>
+      <c r="D4">
+        <v>14.29</v>
+      </c>
+      <c r="E4">
+        <v>84.96</v>
+      </c>
+      <c r="F4">
+        <v>13.4636</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
-      <c r="B6">
-        <v>12.95</v>
-      </c>
-      <c r="C6">
-        <v>88.5</v>
-      </c>
-      <c r="D6">
-        <v>14.41</v>
-      </c>
-      <c r="E6">
-        <v>1569</v>
-      </c>
-      <c r="F6">
-        <v>17.093699999999998</v>
-      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>1</v>
       </c>
-      <c r="B7">
-        <v>6.7</v>
-      </c>
-      <c r="C7">
-        <v>93.81</v>
-      </c>
-      <c r="D7">
-        <v>7.21</v>
-      </c>
-      <c r="E7">
-        <v>1271.3599999999999</v>
-      </c>
-      <c r="F7">
-        <v>240.96270000000001</v>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9" t="s">
-        <v>4</v>
-      </c>
-      <c r="E9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" t="s">
-        <v>9</v>
+        <v>0</v>
+      </c>
+      <c r="B9">
+        <v>22.77</v>
+      </c>
+      <c r="C9">
+        <v>78.38</v>
+      </c>
+      <c r="D9">
+        <v>23.89</v>
+      </c>
+      <c r="E9">
+        <v>2073.16</v>
+      </c>
+      <c r="F9">
+        <v>17.4329</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10">
-        <v>16.96</v>
+        <v>14.8</v>
       </c>
       <c r="C10">
-        <v>78.760000000000005</v>
+        <v>83.93</v>
       </c>
       <c r="D10">
-        <v>12.61</v>
+        <v>13.51</v>
       </c>
       <c r="E10">
-        <v>97.97</v>
+        <v>5619.32</v>
       </c>
       <c r="F10">
-        <v>1.5811999999999999</v>
+        <v>155.00290000000001</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11">
-        <v>13.39</v>
-      </c>
-      <c r="C11">
-        <v>87.5</v>
-      </c>
-      <c r="D11">
-        <v>14.29</v>
-      </c>
-      <c r="E11">
-        <v>84.96</v>
-      </c>
-      <c r="F11">
-        <v>13.4636</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12">
+        <v>27.23</v>
+      </c>
+      <c r="C12">
+        <v>70.8</v>
+      </c>
+      <c r="D12">
+        <v>25.23</v>
+      </c>
+      <c r="E12">
+        <v>2892.71</v>
+      </c>
+      <c r="F12">
+        <v>34.570399999999999</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" t="s">
-        <v>2</v>
-      </c>
-      <c r="C13" t="s">
-        <v>3</v>
-      </c>
-      <c r="D13" t="s">
-        <v>4</v>
-      </c>
-      <c r="E13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" t="s">
-        <v>9</v>
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>16.96</v>
+      </c>
+      <c r="C13">
+        <v>80.53</v>
+      </c>
+      <c r="D13">
+        <v>14.41</v>
+      </c>
+      <c r="E13">
+        <v>5060.3500000000004</v>
+      </c>
+      <c r="F13">
+        <v>78.007099999999994</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15">
+        <v>15</v>
+      </c>
+      <c r="C15">
+        <v>85.32</v>
+      </c>
+      <c r="D15">
+        <v>17.12</v>
+      </c>
+      <c r="E15">
+        <v>289.43</v>
+      </c>
+      <c r="F15">
+        <v>1.4267000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>1</v>
+      </c>
+      <c r="B16">
+        <v>9.82</v>
+      </c>
+      <c r="C16">
+        <v>90.18</v>
+      </c>
+      <c r="D16">
+        <v>9.82</v>
+      </c>
+      <c r="E16">
+        <v>305.13</v>
+      </c>
+      <c r="F16">
+        <v>27.958100000000002</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" t="s">
-        <v>2</v>
-      </c>
-      <c r="C17" t="s">
-        <v>3</v>
-      </c>
-      <c r="D17" t="s">
-        <v>4</v>
-      </c>
-      <c r="E17" t="s">
-        <v>8</v>
-      </c>
-      <c r="F17" t="s">
         <v>9</v>
       </c>
     </row>
@@ -639,19 +626,19 @@
         <v>0</v>
       </c>
       <c r="B18">
-        <v>22.77</v>
+        <v>12.95</v>
       </c>
       <c r="C18">
-        <v>78.38</v>
+        <v>88.5</v>
       </c>
       <c r="D18">
-        <v>23.89</v>
+        <v>14.41</v>
       </c>
       <c r="E18">
-        <v>2073.16</v>
+        <v>1569</v>
       </c>
       <c r="F18">
-        <v>17.4329</v>
+        <v>17.093699999999998</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -659,64 +646,19 @@
         <v>1</v>
       </c>
       <c r="B19">
-        <v>14.8</v>
+        <v>6.7</v>
       </c>
       <c r="C19">
-        <v>83.93</v>
+        <v>93.81</v>
       </c>
       <c r="D19">
-        <v>13.51</v>
+        <v>7.21</v>
       </c>
       <c r="E19">
-        <v>5619.32</v>
+        <v>1271.3599999999999</v>
       </c>
       <c r="F19">
-        <v>155.00290000000001</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B21" t="s">
-        <v>2</v>
-      </c>
-      <c r="C21" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" t="s">
-        <v>4</v>
-      </c>
-      <c r="E21" t="s">
-        <v>8</v>
-      </c>
-      <c r="F21" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B22">
-        <v>27.23</v>
-      </c>
-      <c r="C22">
-        <v>70.8</v>
-      </c>
-      <c r="D22">
-        <v>25.23</v>
-      </c>
-      <c r="E22">
-        <v>2892.71</v>
-      </c>
-      <c r="F22">
-        <v>34.570399999999999</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>1</v>
+        <v>240.96270000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>